<commit_message>
Update prices to real scraped values from all 3 stores
All prices now fetched from actual product pages (Feb 2026).
Previous prices were rough estimates — many were off by 3-10x,
especially hardware, screws, and specialty items.

Notes updated for pack-size differences between stores.
</commit_message>
<xml_diff>
--- a/gate_shopping_list_v3.xlsx
+++ b/gate_shopping_list_v3.xlsx
@@ -730,7 +730,7 @@
     <row r="2" ht="18" customHeight="1" s="29">
       <c r="A2" s="31" t="inlineStr">
         <is>
-          <t>3 stores on Industrivej, Roskilde: Bauhaus (#52) · Silvan (#26) · Jem &amp; Fix (#24)  |  Prices est. Feb 2026</t>
+          <t>3 stores on Industrivej, Roskilde: Bauhaus (#52) · Silvan (#26) · Jem &amp; Fix (#24)  |  Prices scraped Feb 2026</t>
         </is>
       </c>
     </row>
@@ -861,21 +861,21 @@
         </is>
       </c>
       <c r="F5" s="39" t="n">
-        <v>53</v>
+        <v>52.68</v>
       </c>
       <c r="G5" s="39">
         <f>D5*F5</f>
         <v/>
       </c>
       <c r="H5" s="40" t="n">
-        <v>48</v>
+        <v>49.8</v>
       </c>
       <c r="I5" s="40">
         <f>D5*H5</f>
         <v/>
       </c>
       <c r="J5" s="41" t="n">
-        <v>36</v>
+        <v>49.8</v>
       </c>
       <c r="K5" s="41">
         <f>D5*J5</f>
@@ -946,21 +946,21 @@
         </is>
       </c>
       <c r="F7" s="39" t="n">
-        <v>12</v>
+        <v>11.68</v>
       </c>
       <c r="G7" s="39">
         <f>D7*F7</f>
         <v/>
       </c>
       <c r="H7" s="40" t="n">
-        <v>13</v>
+        <v>12.95</v>
       </c>
       <c r="I7" s="40">
         <f>D7*H7</f>
         <v/>
       </c>
       <c r="J7" s="41" t="n">
-        <v>11</v>
+        <v>10.71</v>
       </c>
       <c r="K7" s="41">
         <f>D7*J7</f>
@@ -1031,21 +1031,21 @@
         </is>
       </c>
       <c r="F9" s="39" t="n">
-        <v>12</v>
+        <v>11.68</v>
       </c>
       <c r="G9" s="39">
         <f>D9*F9</f>
         <v/>
       </c>
       <c r="H9" s="40" t="n">
-        <v>13</v>
+        <v>12.95</v>
       </c>
       <c r="I9" s="40">
         <f>D9*H9</f>
         <v/>
       </c>
       <c r="J9" s="41" t="n">
-        <v>11</v>
+        <v>10.71</v>
       </c>
       <c r="K9" s="41">
         <f>D9*J9</f>
@@ -1115,22 +1115,20 @@
           <t>pcs</t>
         </is>
       </c>
-      <c r="F11" s="39" t="n">
-        <v>40</v>
-      </c>
+      <c r="F11" s="39" t="n"/>
       <c r="G11" s="39">
         <f>D11*F11</f>
         <v/>
       </c>
       <c r="H11" s="40" t="n">
-        <v>17</v>
+        <v>16.95</v>
       </c>
       <c r="I11" s="40">
         <f>D11*H11</f>
         <v/>
       </c>
       <c r="J11" s="41" t="n">
-        <v>35</v>
+        <v>32.25</v>
       </c>
       <c r="K11" s="41">
         <f>D11*J11</f>
@@ -1153,7 +1151,7 @@
       </c>
       <c r="O11" s="49" t="inlineStr">
         <is>
-          <t>CUT: 6×~310mm shelves from 2 boards. Drill drainage holes! Fits V70.</t>
+          <t>CUT: 6×~310mm shelves from 2 boards. Drill drainage holes! Fits V70. Bauhaus: exact 15x95x1800 not stocked online — check in store.</t>
         </is>
       </c>
     </row>
@@ -1201,21 +1199,21 @@
         </is>
       </c>
       <c r="F13" s="39" t="n">
-        <v>30</v>
+        <v>79.95</v>
       </c>
       <c r="G13" s="39">
         <f>D13*F13</f>
         <v/>
       </c>
       <c r="H13" s="40" t="n">
-        <v>35</v>
+        <v>104.95</v>
       </c>
       <c r="I13" s="40">
         <f>D13*H13</f>
         <v/>
       </c>
       <c r="J13" s="41" t="n">
-        <v>25</v>
+        <v>59</v>
       </c>
       <c r="K13" s="41">
         <f>D13*J13</f>
@@ -1265,21 +1263,21 @@
         </is>
       </c>
       <c r="F14" s="39" t="n">
-        <v>60</v>
+        <v>144.95</v>
       </c>
       <c r="G14" s="39">
         <f>D14*F14</f>
         <v/>
       </c>
       <c r="H14" s="40" t="n">
-        <v>65</v>
+        <v>83.95</v>
       </c>
       <c r="I14" s="40">
         <f>D14*H14</f>
         <v/>
       </c>
       <c r="J14" s="41" t="n">
-        <v>50</v>
+        <v>141</v>
       </c>
       <c r="K14" s="41">
         <f>D14*J14</f>
@@ -1329,21 +1327,21 @@
         </is>
       </c>
       <c r="F15" s="39" t="n">
-        <v>40</v>
+        <v>179.95</v>
       </c>
       <c r="G15" s="39">
         <f>D15*F15</f>
         <v/>
       </c>
       <c r="H15" s="40" t="n">
-        <v>45</v>
+        <v>124.95</v>
       </c>
       <c r="I15" s="40">
         <f>D15*H15</f>
         <v/>
       </c>
       <c r="J15" s="41" t="n">
-        <v>35</v>
+        <v>24.95</v>
       </c>
       <c r="K15" s="41">
         <f>D15*J15</f>
@@ -1393,21 +1391,21 @@
         </is>
       </c>
       <c r="F16" s="39" t="n">
-        <v>15</v>
+        <v>94.95</v>
       </c>
       <c r="G16" s="39">
         <f>D16*F16</f>
         <v/>
       </c>
       <c r="H16" s="40" t="n">
-        <v>18</v>
+        <v>16.95</v>
       </c>
       <c r="I16" s="40">
         <f>D16*H16</f>
         <v/>
       </c>
       <c r="J16" s="41" t="n">
-        <v>12</v>
+        <v>24.75</v>
       </c>
       <c r="K16" s="41">
         <f>D16*J16</f>
@@ -1430,7 +1428,7 @@
       </c>
       <c r="O16" s="49" t="inlineStr">
         <is>
-          <t>8 brackets total for planter frame corners.</t>
+          <t>8 brackets total. Bauhaus 12-pack (94.95) covers it. Silvan/JF sell singles.</t>
         </is>
       </c>
     </row>
@@ -1457,21 +1455,21 @@
         </is>
       </c>
       <c r="F17" s="39" t="n">
-        <v>89</v>
+        <v>419.95</v>
       </c>
       <c r="G17" s="39">
         <f>D17*F17</f>
         <v/>
       </c>
       <c r="H17" s="40" t="n">
-        <v>99</v>
+        <v>239.95</v>
       </c>
       <c r="I17" s="40">
         <f>D17*H17</f>
         <v/>
       </c>
       <c r="J17" s="41" t="n">
-        <v>79</v>
+        <v>389</v>
       </c>
       <c r="K17" s="41">
         <f>D17*J17</f>
@@ -1521,21 +1519,21 @@
         </is>
       </c>
       <c r="F18" s="39" t="n">
-        <v>69</v>
+        <v>519.95</v>
       </c>
       <c r="G18" s="39">
         <f>D18*F18</f>
         <v/>
       </c>
       <c r="H18" s="40" t="n">
-        <v>75</v>
+        <v>309.95</v>
       </c>
       <c r="I18" s="40">
         <f>D18*H18</f>
         <v/>
       </c>
       <c r="J18" s="41" t="n">
-        <v>59</v>
+        <v>79.95</v>
       </c>
       <c r="K18" s="41">
         <f>D18*J18</f>
@@ -1606,21 +1604,21 @@
         </is>
       </c>
       <c r="F20" s="39" t="n">
-        <v>24</v>
+        <v>23.95</v>
       </c>
       <c r="G20" s="39">
         <f>D20*F20</f>
         <v/>
       </c>
       <c r="H20" s="40" t="n">
-        <v>16</v>
+        <v>16.95</v>
       </c>
       <c r="I20" s="40">
         <f>D20*H20</f>
         <v/>
       </c>
       <c r="J20" s="41" t="n">
-        <v>18</v>
+        <v>18.75</v>
       </c>
       <c r="K20" s="41">
         <f>D20*J20</f>
@@ -1670,21 +1668,21 @@
         </is>
       </c>
       <c r="F21" s="39" t="n">
-        <v>45</v>
+        <v>17.49</v>
       </c>
       <c r="G21" s="39">
         <f>D21*F21</f>
         <v/>
       </c>
       <c r="H21" s="40" t="n">
-        <v>49</v>
+        <v>59.95</v>
       </c>
       <c r="I21" s="40">
         <f>D21*H21</f>
         <v/>
       </c>
       <c r="J21" s="41" t="n">
-        <v>39</v>
+        <v>199</v>
       </c>
       <c r="K21" s="41">
         <f>D21*J21</f>
@@ -1707,7 +1705,7 @@
       </c>
       <c r="O21" s="49" t="inlineStr">
         <is>
-          <t>One per planter corner. Search "jordanker" or "grounding spike" in store.</t>
+          <t>Bauhaus: 4-pack (69.95 total). Silvan: stolpespyd 76x76mm. JF: jordspyd m/holder (expensive — consider alternatives).</t>
         </is>
       </c>
     </row>
@@ -1734,21 +1732,21 @@
         </is>
       </c>
       <c r="F22" s="39" t="n">
-        <v>35</v>
+        <v>149.5</v>
       </c>
       <c r="G22" s="39">
         <f>D22*F22</f>
         <v/>
       </c>
       <c r="H22" s="40" t="n">
-        <v>40</v>
+        <v>97.95</v>
       </c>
       <c r="I22" s="40">
         <f>D22*H22</f>
         <v/>
       </c>
       <c r="J22" s="41" t="n">
-        <v>30</v>
+        <v>84.95</v>
       </c>
       <c r="K22" s="41">
         <f>D22*J22</f>
@@ -1771,7 +1769,7 @@
       </c>
       <c r="O22" s="45" t="inlineStr">
         <is>
-          <t>Loop wire from anchor through box frame. Or use ratchet straps you already own.</t>
+          <t>Bauhaus: 14.95/m (buy 10m). Silvan &amp; JF: 10m rolls. Or use ratchet straps you already own.</t>
         </is>
       </c>
     </row>
@@ -1819,21 +1817,21 @@
         </is>
       </c>
       <c r="F24" s="39" t="n">
-        <v>45</v>
+        <v>499.95</v>
       </c>
       <c r="G24" s="39">
         <f>D24*F24</f>
         <v/>
       </c>
       <c r="H24" s="40" t="n">
-        <v>49</v>
+        <v>359.95</v>
       </c>
       <c r="I24" s="40">
         <f>D24*H24</f>
         <v/>
       </c>
       <c r="J24" s="41" t="n">
-        <v>39</v>
+        <v>219</v>
       </c>
       <c r="K24" s="41">
         <f>D24*J24</f>
@@ -1856,7 +1854,7 @@
       </c>
       <c r="O24" s="49" t="inlineStr">
         <is>
-          <t>Lines inside above shelf — keeps soil off wood. Search "plastfolie bygge" in store.</t>
+          <t>All stores sell larger rolls than needed. JF 2x10m is smallest. Bauhaus 2x50m, Silvan 2x25m. Share leftover with a neighbor.</t>
         </is>
       </c>
     </row>
@@ -1883,21 +1881,21 @@
         </is>
       </c>
       <c r="F25" s="39" t="n">
-        <v>50</v>
+        <v>59.95</v>
       </c>
       <c r="G25" s="39">
         <f>D25*F25</f>
         <v/>
       </c>
       <c r="H25" s="40" t="n">
-        <v>55</v>
+        <v>59.95</v>
       </c>
       <c r="I25" s="40">
         <f>D25*H25</f>
         <v/>
       </c>
       <c r="J25" s="41" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="K25" s="41">
         <f>D25*J25</f>

</xml_diff>

<commit_message>
Fix JF jordanker: use Stavrex skruespids (69 kr) instead of post holder (199 kr)
The previous JF link pointed to a "jordspyd m/holder" which is a post holder
with mount bracket, not a ground anchor. Replaced with Stavrex skruespids
jordskrue Ø25x445mm — an actual ground anchor screw for securing structures.
</commit_message>
<xml_diff>
--- a/gate_shopping_list_v3.xlsx
+++ b/gate_shopping_list_v3.xlsx
@@ -1682,7 +1682,7 @@
         <v/>
       </c>
       <c r="J21" s="41" t="n">
-        <v>199</v>
+        <v>69</v>
       </c>
       <c r="K21" s="41">
         <f>D21*J21</f>
@@ -1700,12 +1700,12 @@
       </c>
       <c r="N21" s="44" t="inlineStr">
         <is>
-          <t>https://www.jemogfix.dk/jordspyd-mholder-galvaniseret-staal/5101/9078974/</t>
+          <t>https://www.jemogfix.dk/stavrex-skruespids-jordskrue-oe25-x-445-mm/5101/9068212/</t>
         </is>
       </c>
       <c r="O21" s="49" t="inlineStr">
         <is>
-          <t>Bauhaus: 4-pack (69.95 total). Silvan: stolpespyd 76x76mm. JF: jordspyd m/holder (expensive — consider alternatives).</t>
+          <t>JF: Stavrex skruespids 445mm (69 kr/stk) — screw into ground next to planter, wire to frame. Bauhaus: 4-pack (69.95 total). Silvan: stolpespyd.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify all JF products and optimize for cheapest options
- Skruer: switch from A4 rustfri (389 kr) to Climate-G3 (103 kr) — saves 286 kr
- Jordanker: switch to stolpespyd 7.1x7.1x75cm (38.75 kr vs 69/199 kr)
- Vinkelbeslag: fix link from category page to specific 40x40x15mm 2-stk product
- Verify all 14 JF product links point to correct products with real prices
- JF total: ~2,511 kr
</commit_message>
<xml_diff>
--- a/gate_shopping_list_v3.xlsx
+++ b/gate_shopping_list_v3.xlsx
@@ -1364,7 +1364,7 @@
       </c>
       <c r="O15" s="45" t="inlineStr">
         <is>
-          <t>Extra toddler lock at gate bottom. JF link is exact product.</t>
+          <t>JF: 150mm elforzinket (24.95 kr). For full outdoor use, consider the 230mm galvaniseret (129 kr). Bottom of gate is somewhat sheltered.</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
         <v/>
       </c>
       <c r="J16" s="41" t="n">
-        <v>24.75</v>
+        <v>19.95</v>
       </c>
       <c r="K16" s="41">
         <f>D16*J16</f>
@@ -1423,12 +1423,12 @@
       </c>
       <c r="N16" s="44" t="inlineStr">
         <is>
-          <t>https://www.jemogfix.dk/beslag-til-havelaage/5109/9045542/</t>
+          <t>https://www.jemogfix.dk/vinkelbeslag-40-x-40-x-15-mm-2-stk/5101/9052892/</t>
         </is>
       </c>
       <c r="O16" s="49" t="inlineStr">
         <is>
-          <t>8 brackets total. Bauhaus 12-pack (94.95) covers it. Silvan/JF sell singles.</t>
+          <t>8 brackets total = 4x 2-packs. JF: 40x40x15mm 2-stk incl. screws. Bauhaus 12-pack (94.95) also covers it.</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1438,7 @@
       </c>
       <c r="B17" s="37" t="inlineStr">
         <is>
-          <t>Skruer rustfri 4.0×40mm (200pk)</t>
+          <t>Skruer Climate-G3 4.0×40mm (200pk)</t>
         </is>
       </c>
       <c r="C17" s="38" t="inlineStr">
@@ -1469,7 +1469,7 @@
         <v/>
       </c>
       <c r="J17" s="41" t="n">
-        <v>389</v>
+        <v>103</v>
       </c>
       <c r="K17" s="41">
         <f>D17*J17</f>
@@ -1487,12 +1487,12 @@
       </c>
       <c r="N17" s="44" t="inlineStr">
         <is>
-          <t>https://www.jemogfix.dk/nkt-fasteners-spunplus-spunskrue-rustfri-a4-4-0-x-40-mm-300-stk/5111/9040074/</t>
+          <t>https://www.jemogfix.dk/nkt-fasteners-spunplus-climate-skrue-4-0-x-40-mm-200-stk/5111/9033433/</t>
         </is>
       </c>
       <c r="O17" s="45" t="inlineStr">
         <is>
-          <t>For cladding, pickets, shelf boards. Search "rustfri skruer 4×40" in store.</t>
+          <t>Climate-G3 coating is outdoor rated (~2000hrs salt spray). A4 rustfri is overkill unless coastal. JF Climate = 103 kr vs 389 kr for A4!</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
         <v/>
       </c>
       <c r="J21" s="41" t="n">
-        <v>69</v>
+        <v>38.75</v>
       </c>
       <c r="K21" s="41">
         <f>D21*J21</f>
@@ -1700,12 +1700,12 @@
       </c>
       <c r="N21" s="44" t="inlineStr">
         <is>
-          <t>https://www.jemogfix.dk/stavrex-skruespids-jordskrue-oe25-x-445-mm/5101/9068212/</t>
+          <t>https://www.jemogfix.dk/stolpespyd-7-1-x-7-1-x-75-cm/5101/9011668/</t>
         </is>
       </c>
       <c r="O21" s="49" t="inlineStr">
         <is>
-          <t>JF: Stavrex skruespids 445mm (69 kr/stk) — screw into ground next to planter, wire to frame. Bauhaus: 4-pack (69.95 total). Silvan: stolpespyd.</t>
+          <t>JF: Stolpespyd 7.1x7.1x75cm (38.75 kr/stk) — drive into ground, wire to planter frame. Bauhaus: 4-pack (69.95 total). Silvan: stolpespyd 76x76mm.</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" display="https://www.jemogfix.dk/skudrigle-150-mm/5109/9052891/" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" display="https://www.jemogfix.dk/beslag-til-havelaage/5109/9045542/" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId27"/>

</xml_diff>

<commit_message>
Update to 3.5m span with 115cm wide planters
Measured actual space at 3.5m across. Planters widened from 40cm to 115cm
(350 - 120 gate) / 2 = 115cm each.

Changes:
- index.html: Updated all geometry builders, step descriptions, materials
  quantities, camera positions for wider scene
- viewer.html: Updated planter width, positions, dynamic cladding/shelf
  board counts, ballast to 3 slabs, camera zoom
- README.md: Updated planter dimensions
- Excel: Updated quantities (cladding 56, shelf boards 4, soil 6 bags, etc.)
</commit_message>
<xml_diff>
--- a/gate_shopping_list_v3.xlsx
+++ b/gate_shopping_list_v3.xlsx
@@ -723,7 +723,7 @@
     <row r="1" ht="27.75" customHeight="1" s="29">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>PLANTER BOX GATE — Complete Shopping List (120cm tall)</t>
+          <t>PLANTER BOX GATE — Complete Shopping List (3.5m span, 115cm planters, 120cm tall)</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
       </c>
       <c r="O5" s="45" t="inlineStr">
         <is>
-          <t>CUT: 1×1200mm + 1×1200mm per board (zero waste!). Shortest stocked length = 2400mm. Sticks out ~60cm in V70 with tailgate open — tie a red flag on it.</t>
+          <t>CUT PLAN CHANGED: Posts 8×1200mm (4 boards). Width rails 12×1060mm (6 boards, 2 per board). Depth rails 12×210mm (from offcuts). Gate 3 boards. Total ~15.</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="D7" s="46" t="n">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="E7" s="46" t="inlineStr">
         <is>
@@ -983,7 +983,7 @@
       </c>
       <c r="O7" s="49" t="inlineStr">
         <is>
-          <t>CUT: each to 1200mm. 4 faces × 3 boards × 2 boxes = 24. These fit the V70 perfectly at 1800mm.</t>
+          <t>CUT: each to 1200mm. With 115cm planters: front/back need 11 boards each, sides need 3 each. 2×(2×11 + 2×3) = 56 boards.</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="D11" s="46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E11" s="46" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="O11" s="49" t="inlineStr">
         <is>
-          <t>CUT: 6×~310mm shelves from 2 boards. Drill drainage holes! Fits V70. Bauhaus: exact 15x95x1800 not stocked online — check in store.</t>
+          <t>Boards span depth (210mm), laid across 1060mm width. ~12 per planter = 24 pieces. Cut 8 per 1800mm board. Need 4 boards. Bauhaus: exact 15x95x1800 not stocked online.</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="D17" s="36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" s="36" t="inlineStr">
         <is>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="O17" s="45" t="inlineStr">
         <is>
-          <t>Climate-G3 coating is outdoor rated (~2000hrs salt spray). A4 rustfri is overkill unless coastal. JF Climate = 103 kr vs 389 kr for A4!</t>
+          <t>56 cladding boards + 14 pickets + shelves ≈ 400 screws. Need 2× 200-packs. Climate-G3 is outdoor rated.</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1596,7 @@
         </is>
       </c>
       <c r="D20" s="36" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E20" s="36" t="inlineStr">
         <is>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="O20" s="45" t="inlineStr">
         <is>
-          <t>4 under boxes (base) + 4 inside (ballast, ~30kg). JF/Silvan: search "betonflise 40x40" in store.</t>
+          <t>Base: 3 per planter (covers 120cm width). Ballast inside: 3 per planter. Total 12.</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="D25" s="36" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E25" s="36" t="inlineStr">
         <is>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="O25" s="45" t="inlineStr">
         <is>
-          <t>~40L per box. Plant herbs, strawberries, flowers!</t>
+          <t>~111L soil per planter with 115cm width. 6× 40L bags = 240L total.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix forskallingsbræt: 3000mm boards (not 1800mm), qty 4→2
JF sells imp. høvlet 15×95×3000mm at 32.25 kr. Each 3m board yields
~14 pieces of 210mm, so only 2 boards needed for 24 shelf pieces.

- Updated Excel item name, qty, links for all 3 stores
- Cleared Bauhaus/Silvan prices (unverified for this product)
- Updated index.html step 4 instructions to match
</commit_message>
<xml_diff>
--- a/gate_shopping_list_v3.xlsx
+++ b/gate_shopping_list_v3.xlsx
@@ -1099,7 +1099,7 @@
       </c>
       <c r="B11" s="47" t="inlineStr">
         <is>
-          <t>Forskallingsbræt 15×95×1800mm høvl.</t>
+          <t>Imp. høvlet bræt 15×95×3000mm</t>
         </is>
       </c>
       <c r="C11" s="48" t="inlineStr">
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="D11" s="46" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E11" s="46" t="inlineStr">
         <is>
@@ -1120,9 +1120,7 @@
         <f>D11*F11</f>
         <v/>
       </c>
-      <c r="H11" s="40" t="n">
-        <v>16.95</v>
-      </c>
+      <c r="H11" s="40" t="n"/>
       <c r="I11" s="40">
         <f>D11*H11</f>
         <v/>
@@ -1136,12 +1134,12 @@
       </c>
       <c r="L11" s="42" t="inlineStr">
         <is>
-          <t>https://www.bauhaus.dk/froeslev-forskalling-hoevlet-flere-stoerrelser</t>
+          <t>https://www.bauhaus.dk/froslev-hegnsbraedder-hovlet-19x100x3000-mm-15x95-mm</t>
         </is>
       </c>
       <c r="M11" s="43" t="inlineStr">
         <is>
-          <t>https://www.silvan.dk/produkt/froeslev-forskallingsbraet-15x95x1800-mm-trykimpraegneret-hoevlet-7710-9421711</t>
+          <t>https://www.silvan.dk/produkt/froeslev-forskallingsbraet-15x95x3000-mm-trykimpraegneret-hoevlet-7710-9441492</t>
         </is>
       </c>
       <c r="N11" s="44" t="inlineStr">
@@ -2106,7 +2104,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" display="https://www.silvan.dk/ft-braedder-trykimpraegneret-gran-100-mm-1800-mm-16-mm?id=7710-9805872" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" display="https://www.jemogfix.dk/imp-ru-braedder-16-x-100-x-1800-mm/4310/9057351/" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" display="https://www.silvan.dk/produkt/froeslev-forskallingsbraet-15x95x1800-mm-trykimpraegneret-hoevlet-7710-9421711" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" display="https://www.bauhaus.dk/pn-t-haengsel-12-galvaniseret-310-mm" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId14"/>

</xml_diff>

<commit_message>
Fix skudrigle: 160mm at 64.95 kr (was wrong 150mm at 24.95 kr)
JF doesn't sell a 150mm skudrigle. Updated to 160mm elforzinket
at 64.95 kr with correct product link.
</commit_message>
<xml_diff>
--- a/gate_shopping_list_v3.xlsx
+++ b/gate_shopping_list_v3.xlsx
@@ -1308,7 +1308,7 @@
       </c>
       <c r="B15" s="37" t="inlineStr">
         <is>
-          <t>Skudrigle 150mm galvaniseret</t>
+          <t>Skudrigle 160mm elforzinket</t>
         </is>
       </c>
       <c r="C15" s="38" t="inlineStr">
@@ -1339,7 +1339,7 @@
         <v/>
       </c>
       <c r="J15" s="41" t="n">
-        <v>24.95</v>
+        <v>64.95</v>
       </c>
       <c r="K15" s="41">
         <f>D15*J15</f>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="N15" s="44" t="inlineStr">
         <is>
-          <t>https://www.jemogfix.dk/skudrigle-150-mm/5109/9052891/</t>
+          <t>https://www.jemogfix.dk/skudrigle-160-mm/5109/9052888/</t>
         </is>
       </c>
       <c r="O15" s="45" t="inlineStr">
@@ -2114,7 +2114,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" display="https://www.jemogfix.dk/stalddoersgreb-til-doere-paa-40-90-mm/5100/9052881/" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" display="https://www.jemogfix.dk/skudrigle-150-mm/5109/9052891/" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId24"/>

</xml_diff>